<commit_message>
bulk excel uploaded and role based response changed
</commit_message>
<xml_diff>
--- a/hostel_management_Frontend/public/sample2.xlsx
+++ b/hostel_management_Frontend/public/sample2.xlsx
@@ -27,88 +27,104 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
   <si>
     <t>s.no</t>
   </si>
   <si>
-    <t>Location</t>
-  </si>
-  <si>
-    <t>Gate</t>
-  </si>
-  <si>
-    <t>Product Type</t>
-  </si>
-  <si>
-    <t>Vehicle Number</t>
-  </si>
-  <si>
-    <t>Vehicle Rfid</t>
-  </si>
-  <si>
-    <t>Vehicle status</t>
+    <t>Member ID</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>Degree</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Expiry Date</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Hostel Name</t>
+  </si>
+  <si>
+    <t>Room No</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>Parant/Guardian Name</t>
+  </si>
+  <si>
+    <t>Parant/Guardian Contact</t>
   </si>
   <si>
     <t>Remark</t>
   </si>
   <si>
-    <t>Casa grand oragadam</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Gate 1</t>
-  </si>
-  <si>
-    <t>Car</t>
-  </si>
-  <si>
-    <t>tn33h6332</t>
-  </si>
-  <si>
-    <t>214090129d89409002928489</t>
-  </si>
-  <si>
-    <t>Active</t>
+    <t>2cqr automation</t>
+  </si>
+  <si>
+    <t>Computer science</t>
+  </si>
+  <si>
+    <t>B.com</t>
+  </si>
+  <si>
+    <t>2cqr1@gmail.com</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>srm girls hostel</t>
+  </si>
+  <si>
+    <t>chennai</t>
+  </si>
+  <si>
+    <t>arun</t>
   </si>
   <si>
     <t>Remarks</t>
   </si>
   <si>
-    <t>tndsfbh6332</t>
-  </si>
-  <si>
-    <t>224090129d89409002928489</t>
-  </si>
-  <si>
-    <t>tn113bh6332</t>
-  </si>
-  <si>
-    <t>304092129d89409002928489</t>
-  </si>
-  <si>
-    <t>tn213bh6332</t>
-  </si>
-  <si>
-    <t>244090129d89409002928489</t>
-  </si>
-  <si>
-    <t>tnb213h6332</t>
-  </si>
-  <si>
-    <t>254090129d89409002928489</t>
+    <t>2cqr pvt</t>
+  </si>
+  <si>
+    <t>Commerce</t>
+  </si>
+  <si>
+    <t>Bsc</t>
+  </si>
+  <si>
+    <t>Female</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="180" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -117,10 +133,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -128,14 +145,6 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -583,162 +592,162 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6"/>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1058,173 +1067,162 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5" outlineLevelCol="7"/>
+  <dimension ref="A1:O3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
-    <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="6" width="17.6296296296296" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.1759259259259" style="1" customWidth="1"/>
-    <col min="8" max="8" width="12.9074074074074" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="1"/>
+    <col min="2" max="9" width="17.6296296296296" customWidth="1"/>
+    <col min="10" max="14" width="15.1759259259259" customWidth="1"/>
+    <col min="15" max="15" width="12.9074074074074" customWidth="1"/>
+    <col min="16" max="16" width="15.1759259259259" customWidth="1"/>
+    <col min="17" max="17" width="12.9074074074074" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:8">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="1" ht="28.8" spans="1:15">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:8">
-      <c r="A2" s="1">
+    <row r="2" customFormat="1" spans="1:15">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>14</v>
+      <c r="B2">
+        <v>567</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2">
+        <v>9791344113</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" s="4">
+        <v>46016</v>
+      </c>
+      <c r="I2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2">
+        <v>100</v>
+      </c>
+      <c r="L2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N2">
+        <v>9791344113</v>
+      </c>
+      <c r="O2" t="s">
+        <v>23</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:8">
-      <c r="A3" s="1">
+    <row r="3" customFormat="1" spans="1:15">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" s="1" customFormat="1" spans="1:8">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="5" t="s">
+      <c r="B3">
+        <v>789</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3">
+        <v>9791344112</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" s="1" customFormat="1" spans="1:8">
-      <c r="A5" s="1">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="5" t="s">
+      <c r="H3" s="4">
+        <v>46016</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" s="1" customFormat="1" spans="1:8">
-      <c r="A6" s="1">
-        <v>1</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="1" t="s">
+      <c r="K3">
+        <v>100</v>
+      </c>
+      <c r="L3" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="M3" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>14</v>
+      <c r="N3">
+        <v>9791344113</v>
+      </c>
+      <c r="O3" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" display="2cqr1@gmail.com"/>
+    <hyperlink ref="G3" r:id="rId1" display="2cqr1@gmail.com"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="256" orientation="portrait" horizontalDpi="203" verticalDpi="203"/>
   <headerFooter/>

</xml_diff>